<commit_message>
XML and .md extractors added
</commit_message>
<xml_diff>
--- a/data/knowledge_base/mcq_knowledge_base.xlsx
+++ b/data/knowledge_base/mcq_knowledge_base.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1036"/>
+  <dimension ref="A1:T1043"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -63017,6 +63017,492 @@
       <c r="S1036" t="inlineStr"/>
       <c r="T1036" t="inlineStr"/>
     </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>df844b31-3f70-4e09-ae1e-95b9a5a3c5d7</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>What is the primary purpose of backpropagation in neural networks?</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>To forward propagate inputs through the network</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>To calculate gradients and update weights</t>
+        </is>
+      </c>
+      <c r="E1037" t="inlineStr">
+        <is>
+          <t>To initialize network parameters</t>
+        </is>
+      </c>
+      <c r="F1037" t="inlineStr">
+        <is>
+          <t>To evaluate model performance</t>
+        </is>
+      </c>
+      <c r="G1037" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H1037" t="inlineStr"/>
+      <c r="I1037" t="inlineStr"/>
+      <c r="J1037" t="inlineStr"/>
+      <c r="K1037" t="inlineStr"/>
+      <c r="L1037" t="inlineStr">
+        <is>
+          <t>test_sample.py</t>
+        </is>
+      </c>
+      <c r="M1037" t="inlineStr">
+        <is>
+          <t>2026-07-10 23:34:39</t>
+        </is>
+      </c>
+      <c r="N1037" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1037" t="inlineStr"/>
+      <c r="P1037" t="inlineStr"/>
+      <c r="Q1037" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1037" t="inlineStr"/>
+      <c r="S1037" t="inlineStr"/>
+      <c r="T1037" t="inlineStr"/>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>253f8647-4de4-4f53-a8a2-b6df1cd7aefa</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Which algorithm is used for dimensionality reduction?</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>K-means clustering</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>Linear Regression</t>
+        </is>
+      </c>
+      <c r="E1038" t="inlineStr">
+        <is>
+          <t>Principal Component Analysis (PCA)</t>
+        </is>
+      </c>
+      <c r="F1038" t="inlineStr">
+        <is>
+          <t>Decision Trees</t>
+        </is>
+      </c>
+      <c r="G1038" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H1038" t="inlineStr"/>
+      <c r="I1038" t="inlineStr"/>
+      <c r="J1038" t="inlineStr"/>
+      <c r="K1038" t="inlineStr"/>
+      <c r="L1038" t="inlineStr">
+        <is>
+          <t>test_sample.py</t>
+        </is>
+      </c>
+      <c r="M1038" t="inlineStr">
+        <is>
+          <t>2026-07-10 23:34:39</t>
+        </is>
+      </c>
+      <c r="N1038" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1038" t="inlineStr"/>
+      <c r="P1038" t="inlineStr"/>
+      <c r="Q1038" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1038" t="inlineStr"/>
+      <c r="S1038" t="inlineStr"/>
+      <c r="T1038" t="inlineStr"/>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>655da07f-554b-4e4c-9945-1090c61c97a7</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>In a distributed system, what is the CAP theorem?</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Consistency, Availability, Partition tolerance</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>Caching, API, Performance</t>
+        </is>
+      </c>
+      <c r="E1039" t="inlineStr">
+        <is>
+          <t>Centralization, Authentication, Privacy</t>
+        </is>
+      </c>
+      <c r="F1039" t="inlineStr">
+        <is>
+          <t>Clustering, Aggregation, Partitioning</t>
+        </is>
+      </c>
+      <c r="G1039" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H1039" t="inlineStr"/>
+      <c r="I1039" t="inlineStr"/>
+      <c r="J1039" t="inlineStr"/>
+      <c r="K1039" t="inlineStr"/>
+      <c r="L1039" t="inlineStr">
+        <is>
+          <t>test_sample.py</t>
+        </is>
+      </c>
+      <c r="M1039" t="inlineStr">
+        <is>
+          <t>2026-07-10 23:34:39</t>
+        </is>
+      </c>
+      <c r="N1039" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1039" t="inlineStr"/>
+      <c r="P1039" t="inlineStr"/>
+      <c r="Q1039" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1039" t="inlineStr"/>
+      <c r="S1039" t="inlineStr"/>
+      <c r="T1039" t="inlineStr"/>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>3b61a0d3-53ea-4043-a59d-46cc30471abb</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>What is the primary purpose of backpropagation in neural networks?</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>To forward propagate inputs through the network</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>To calculate gradients and update weights</t>
+        </is>
+      </c>
+      <c r="E1040" t="inlineStr">
+        <is>
+          <t>To initialize network parameters</t>
+        </is>
+      </c>
+      <c r="F1040" t="inlineStr">
+        <is>
+          <t>To evaluate model performance</t>
+        </is>
+      </c>
+      <c r="G1040" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="H1040" t="inlineStr"/>
+      <c r="I1040" t="inlineStr">
+        <is>
+          <t>Conceptual</t>
+        </is>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>ML</t>
+        </is>
+      </c>
+      <c r="K1040" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L1040" t="inlineStr">
+        <is>
+          <t>test_sample.py</t>
+        </is>
+      </c>
+      <c r="M1040" t="inlineStr">
+        <is>
+          <t>2026-07-10 23:34:50</t>
+        </is>
+      </c>
+      <c r="N1040" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1040" t="inlineStr"/>
+      <c r="P1040" t="inlineStr"/>
+      <c r="Q1040" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1040" t="inlineStr"/>
+      <c r="S1040" t="inlineStr"/>
+      <c r="T1040" t="inlineStr"/>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>c70d118d-d427-4ffc-ad76-28dff1d7e10e</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Which algorithm is used for dimensionality reduction?</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>K-means clustering</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>Linear Regression</t>
+        </is>
+      </c>
+      <c r="E1041" t="inlineStr">
+        <is>
+          <t>Principal Component Analysis (PCA)</t>
+        </is>
+      </c>
+      <c r="F1041" t="inlineStr">
+        <is>
+          <t>Decision Trees</t>
+        </is>
+      </c>
+      <c r="G1041" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H1041" t="inlineStr"/>
+      <c r="I1041" t="inlineStr">
+        <is>
+          <t>Conceptual</t>
+        </is>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="K1041" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="L1041" t="inlineStr">
+        <is>
+          <t>test_sample.py</t>
+        </is>
+      </c>
+      <c r="M1041" t="inlineStr">
+        <is>
+          <t>2026-07-10 23:34:50</t>
+        </is>
+      </c>
+      <c r="N1041" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1041" t="inlineStr"/>
+      <c r="P1041" t="inlineStr"/>
+      <c r="Q1041" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1041" t="inlineStr"/>
+      <c r="S1041" t="inlineStr"/>
+      <c r="T1041" t="inlineStr"/>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>6a6b6060-b906-4343-8d13-3a14920b5a48</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>In a distributed system, what is the CAP theorem?</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Consistency, Availability, Partition tolerance</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>Caching, API, Performance</t>
+        </is>
+      </c>
+      <c r="E1042" t="inlineStr">
+        <is>
+          <t>Centralization, Authentication, Privacy</t>
+        </is>
+      </c>
+      <c r="F1042" t="inlineStr">
+        <is>
+          <t>Clustering, Aggregation, Partitioning</t>
+        </is>
+      </c>
+      <c r="G1042" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H1042" t="inlineStr"/>
+      <c r="I1042" t="inlineStr">
+        <is>
+          <t>Conceptual</t>
+        </is>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>System Design</t>
+        </is>
+      </c>
+      <c r="K1042" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L1042" t="inlineStr">
+        <is>
+          <t>test_sample.py</t>
+        </is>
+      </c>
+      <c r="M1042" t="inlineStr">
+        <is>
+          <t>2026-07-10 23:34:50</t>
+        </is>
+      </c>
+      <c r="N1042" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1042" t="inlineStr"/>
+      <c r="P1042" t="inlineStr"/>
+      <c r="Q1042" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1042" t="inlineStr"/>
+      <c r="S1042" t="inlineStr"/>
+      <c r="T1042" t="inlineStr"/>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>4630b440-6a87-44f4-8f59-12cb52b74b8a</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>When designing a high-throughput distributed system, how does deploying a reverse proxy like NGINX impact overall network latency and load balancing trade-offs across application servers?</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>It compresses static content, balances requests, and offloads SSL termination tasks.</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>It functions as an in-memory key-value cache to store session attributes.</t>
+        </is>
+      </c>
+      <c r="E1043" t="inlineStr">
+        <is>
+          <t>It acts as an asynchronous scheduler to coordinate machine learning training.</t>
+        </is>
+      </c>
+      <c r="F1043" t="inlineStr">
+        <is>
+          <t>It executes complex relational database transactions to ensure consistency.</t>
+        </is>
+      </c>
+      <c r="G1043" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H1043" t="inlineStr">
+        <is>
+          <t>Option B is correct because NGINX compresses static content, balances requests across application servers, and offloads SSL termination tasks. Options A, C, and D are incorrect because they describe functionalities that do not pertain to the primary role of a reverse proxy like NGINX.</t>
+        </is>
+      </c>
+      <c r="I1043" t="inlineStr">
+        <is>
+          <t>Application</t>
+        </is>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>System Design</t>
+        </is>
+      </c>
+      <c r="K1043" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L1043" t="inlineStr">
+        <is>
+          <t>data\processed\test_manual_draft.xml</t>
+        </is>
+      </c>
+      <c r="M1043" t="inlineStr">
+        <is>
+          <t>2026-07-11 01:42:44</t>
+        </is>
+      </c>
+      <c r="N1043" t="n">
+        <v>0</v>
+      </c>
+      <c r="O1043" t="inlineStr"/>
+      <c r="P1043" t="inlineStr"/>
+      <c r="Q1043" t="n">
+        <v>0</v>
+      </c>
+      <c r="R1043" t="inlineStr"/>
+      <c r="S1043" t="inlineStr"/>
+      <c r="T1043" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>